<commit_message>
Updated part lists "Elektrobox_Rahmen.xlsx"
</commit_message>
<xml_diff>
--- a/Stuecklisten/Stueckliste_Elektrobox_Rahmen.xlsx
+++ b/Stuecklisten/Stueckliste_Elektrobox_Rahmen.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\HTL_Bulme\SPL_Project_Watermelon\CandyMachine_Watermelon\Stuecklisten\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E3F7D65-A72E-4B25-8D6F-7D8B044C10B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1D93D1E-75D9-476C-9FC8-CBF40D65CA6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{797F69E5-6349-40C8-ABC7-0C572E2B2F92}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
   <si>
     <t>Anzahl</t>
   </si>
@@ -111,6 +111,15 @@
   </si>
   <si>
     <t>5x Corner brackets</t>
+  </si>
+  <si>
+    <t>Stahlblech verzinkt</t>
+  </si>
+  <si>
+    <t>https://www.grosschaedl.at/</t>
+  </si>
+  <si>
+    <t>625x110x0,55mm</t>
   </si>
 </sst>
 </file>
@@ -188,8 +197,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{B9A48411-3BEC-4BB6-80B7-9F4291AC7A73}" name="Tabelle1" displayName="Tabelle1" ref="A1:G7" totalsRowShown="0">
-  <autoFilter ref="A1:G7" xr:uid="{B9A48411-3BEC-4BB6-80B7-9F4291AC7A73}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{B9A48411-3BEC-4BB6-80B7-9F4291AC7A73}" name="Tabelle1" displayName="Tabelle1" ref="A1:G8" totalsRowShown="0">
+  <autoFilter ref="A1:G8" xr:uid="{B9A48411-3BEC-4BB6-80B7-9F4291AC7A73}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{B195A8D2-EFFF-4219-934E-FECCD6DF88AA}" name="Anzahl"/>
     <tableColumn id="2" xr3:uid="{65152C0F-D7FB-4DF5-9078-F76FDC6C07C4}" name="Link (URL)" dataCellStyle="Link"/>
@@ -522,7 +531,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{873408D1-FEA1-4C01-9395-0C80F48BC176}">
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="11" customWidth="1"/>
@@ -697,6 +706,30 @@
       </c>
       <c r="G7" t="s">
         <v>22</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A8">
+        <v>1</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C8" s="1">
+        <v>17.91</v>
+      </c>
+      <c r="D8" t="s">
+        <v>25</v>
+      </c>
+      <c r="E8">
+        <v>223323200</v>
+      </c>
+      <c r="F8" s="1">
+        <f>A8*C8</f>
+        <v>17.91</v>
+      </c>
+      <c r="G8" t="s">
+        <v>27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>